<commit_message>
Correct device transfers in LUCAS3 battery plan
Two corrections to the equipment moves the plan is built on:

- R7: 救急犬山1's vehicle was renewed with no LUCAS purchase; 救急犬山4's
  unit (with its R3/R6 batteries) was transferred to it, leaving 救急犬山4
  with no device until R9.
- R9: the unit freed by 救急犬山2's equipment renewal goes to 救急犬山4,
  not to 救急犬山1.

Re-running the year-by-year ledger under the corrected premise leaves both
totals unchanged — 6 batteries for the 3-year version (R10, R11, R15, R17,
R18, R19) and 3 for the 4-year version (R11 x1, R18 x2), with R9 still at
zero — but the per-vehicle assignments and transfer steps differ. Reference
figures without cross-vehicle swaps stay at 12 and 5, with different years.

Equipment renewal and maintenance inspection years are unchanged from the
source document.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AQM4furAyhVoQYyp8S8kDY
</commit_message>
<xml_diff>
--- a/docs/lucas_battery_plan/犬山市_LUCAS3バッテリ更新計画_R9修正.xlsx
+++ b/docs/lucas_battery_plan/犬山市_LUCAS3バッテリ更新計画_R9修正.xlsx
@@ -114,12 +114,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFE699"/>
+        <fgColor rgb="00E2EFDA"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E2EFDA"/>
+        <fgColor rgb="00FFE699"/>
       </patternFill>
     </fill>
     <fill>
@@ -235,121 +235,121 @@
     <xf numFmtId="0" fontId="8" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -361,10 +361,10 @@
     <xf numFmtId="0" fontId="8" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -378,7 +378,7 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="5" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -787,7 +787,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>元資料「保守点検及び本体、バッテリ更新計画（2026.5修正）」の R9「予備3個購入」を見直したもの。機器更新・保守点検のスケジュールは元資料のまま変更していない。</t>
+          <t>元資料「保守点検及び本体、バッテリ更新計画（2026.5修正）」の R9「予備3個購入」を見直したもの。R7の救急犬山1の車両更新（ルーカス購入なし・救急犬山4の本体を載せ替え）と、救急犬山2の旧本体の載せ替え先が救急犬山4であることを反映。機器更新・保守点検の年度は元資料のまま変更していない。</t>
         </is>
       </c>
     </row>
@@ -1116,19 +1116,19 @@
         <v>0</v>
       </c>
       <c r="O8" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="P8" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="P8" s="12" t="n">
+      <c r="Q8" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="R8" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="S8" s="12" t="n">
         <v>2</v>
-      </c>
-      <c r="Q8" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="R8" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="S8" s="12" t="n">
-        <v>3</v>
       </c>
       <c r="T8" s="13">
         <f>SUM(I8:S8)</f>
@@ -1180,10 +1180,10 @@
         <v>0</v>
       </c>
       <c r="N9" s="12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O9" s="12" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P9" s="12" t="n">
         <v>0</v>
@@ -1192,10 +1192,10 @@
         <v>1</v>
       </c>
       <c r="R9" s="12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S9" s="12" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T9" s="13">
         <f>SUM(I9:S9)</f>
@@ -1637,7 +1637,7 @@
     <row r="19">
       <c r="A19" s="25" t="inlineStr">
         <is>
-          <t>・R9（令和9年度）の予備バッテリ購入は、3年維持版・4年維持版のいずれも 0個。救急犬山2の機器更新（車両更新）で新品バッテリ2個が付属するため。</t>
+          <t>・R9（令和9年度）の予備バッテリ購入は、3年維持版・4年維持版のいずれも 0個。救急犬山2の機器更新（車両更新）で新品バッテリ2個が付属し、旧救急犬山2本体（バッテリ2個付き）が救急犬山4へ回るため。</t>
         </is>
       </c>
     </row>
@@ -1658,7 +1658,7 @@
     <row r="22">
       <c r="A22" s="25" t="inlineStr">
         <is>
-          <t>・本表は元資料の機器更新・保守点検スケジュールを一切変更していない。変更点は予備バッテリの購入年度と個数のみ。</t>
+          <t>・機器更新・保守点検の年度は元資料から一切変更していない。変更点は、本体の載せ替え先（R7＝救4→救1、R9＝旧救2→救4）と、予備バッテリの購入年度・個数のみ。</t>
         </is>
       </c>
     </row>
@@ -1717,7 +1717,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>元資料「保守点検及び本体、バッテリ更新計画（2026.5修正）」の機器更新・保守点検スケジュールはそのまま、R9以降の予備バッテリ購入数のみ精査したもの。</t>
+          <t>元資料「保守点検及び本体、バッテリ更新計画（2026.5修正）」をベースに、①R7の救急犬山1の車両更新（ルーカスは購入せず救急犬山4の本体を載せ替え）、②救急犬山2の旧本体の載せ替え先は救急犬山4、の2点を反映し、R9以降の予備バッテリ購入数を精査したもの。機器更新・保守点検の年度は元資料から変更していない。</t>
         </is>
       </c>
     </row>
@@ -1915,37 +1915,42 @@
       <c r="D7" s="10" t="n"/>
       <c r="E7" s="10" t="n"/>
       <c r="F7" s="10" t="n"/>
-      <c r="G7" s="10" t="n"/>
+      <c r="G7" s="31" t="inlineStr">
+        <is>
+          <t>車両更新（ルーカス購入なし）
+救4の本体を載せ替え（電池R3・R6も）</t>
+        </is>
+      </c>
       <c r="H7" s="10" t="n"/>
-      <c r="I7" s="31" t="inlineStr">
-        <is>
-          <t>旧救2本体を引継（電池R7・R3も引継）</t>
-        </is>
-      </c>
-      <c r="J7" s="32" t="inlineStr">
-        <is>
-          <t>予備1個購入→搭載（R3降ろす）</t>
-        </is>
-      </c>
+      <c r="I7" s="32" t="inlineStr">
+        <is>
+          <t>救2の新品1個を受領（R3降ろす）</t>
+        </is>
+      </c>
+      <c r="J7" s="12" t="n"/>
       <c r="K7" s="12" t="n"/>
-      <c r="L7" s="12" t="n"/>
-      <c r="M7" s="33" t="inlineStr">
-        <is>
-          <t>救2保守点検の新品を搭載（R7降ろす）</t>
-        </is>
-      </c>
-      <c r="N7" s="12" t="n"/>
+      <c r="L7" s="32" t="inlineStr">
+        <is>
+          <t>旧救3本体のR11を受領（R6降ろす）</t>
+        </is>
+      </c>
+      <c r="M7" s="12" t="n"/>
+      <c r="N7" s="32" t="inlineStr">
+        <is>
+          <t>旧救4本体のR13を受領（R9降ろす）</t>
+        </is>
+      </c>
       <c r="O7" s="12" t="n"/>
-      <c r="P7" s="33" t="inlineStr">
-        <is>
-          <t>救3保守点検の新品を搭載（R10降ろす）</t>
+      <c r="P7" s="32" t="inlineStr">
+        <is>
+          <t>救3保守点検の新品を搭載（R11降ろす）</t>
         </is>
       </c>
       <c r="Q7" s="12" t="n"/>
       <c r="R7" s="12" t="n"/>
-      <c r="S7" s="32" t="inlineStr">
-        <is>
-          <t>予備1個購入→搭載（R13降ろす）</t>
+      <c r="S7" s="33" t="inlineStr">
+        <is>
+          <t>予備1個購入→搭載（R16降ろす）</t>
         </is>
       </c>
       <c r="T7" s="12" t="n"/>
@@ -1961,22 +1966,26 @@
       <c r="D8" s="35" t="n"/>
       <c r="E8" s="35" t="n"/>
       <c r="F8" s="35" t="n"/>
-      <c r="G8" s="35" t="n"/>
-      <c r="H8" s="35" t="n"/>
+      <c r="G8" s="35" t="n">
+        <v>6</v>
+      </c>
+      <c r="H8" s="35" t="n">
+        <v>6</v>
+      </c>
       <c r="I8" s="36" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="J8" s="36" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="K8" s="36" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="L8" s="36" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="M8" s="36" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="N8" s="36" t="n">
         <v>13</v>
@@ -2009,28 +2018,32 @@
       <c r="D9" s="37" t="n"/>
       <c r="E9" s="37" t="n"/>
       <c r="F9" s="37" t="n"/>
-      <c r="G9" s="37" t="n"/>
-      <c r="H9" s="37" t="n"/>
+      <c r="G9" s="37" t="n">
+        <v>3</v>
+      </c>
+      <c r="H9" s="37" t="n">
+        <v>3</v>
+      </c>
       <c r="I9" s="38" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="J9" s="38" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="K9" s="38" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="L9" s="38" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="M9" s="38" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="N9" s="38" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="O9" s="38" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="P9" s="38" t="n">
         <v>13</v>
@@ -2074,8 +2087,8 @@
       <c r="I10" s="40" t="n">
         <v>0</v>
       </c>
-      <c r="J10" s="41" t="n">
-        <v>1</v>
+      <c r="J10" s="40" t="n">
+        <v>0</v>
       </c>
       <c r="K10" s="40" t="n">
         <v>0</v>
@@ -2138,34 +2151,35 @@
       <c r="I11" s="31" t="inlineStr">
         <is>
           <t>機器更新（車両更新・電池2個付属）
-新品1個を救4のR6と交換</t>
+旧本体を救4へ／新品1個を救1のR3と交換</t>
         </is>
       </c>
       <c r="J11" s="12" t="n"/>
       <c r="K11" s="12" t="n"/>
-      <c r="L11" s="33" t="inlineStr">
-        <is>
-          <t>救3更新の新品1個を受領（R6降ろす）</t>
+      <c r="L11" s="32" t="inlineStr">
+        <is>
+          <t>救3更新の新品1個を受領（R3降ろす）</t>
         </is>
       </c>
       <c r="M11" s="43" t="inlineStr">
         <is>
-          <t>保守点検（新品1個）→救1へ</t>
+          <t>保守点検（新品1個）→救4へ</t>
         </is>
       </c>
       <c r="N11" s="12" t="n"/>
       <c r="O11" s="32" t="inlineStr">
         <is>
-          <t>予備1個購入→搭載（R9降ろす）</t>
+          <t>救4の新品予備1個を受領
+（救2のR9を救4へ）</t>
         </is>
       </c>
       <c r="P11" s="12" t="n"/>
-      <c r="Q11" s="12" t="n"/>
-      <c r="R11" s="32" t="inlineStr">
+      <c r="Q11" s="33" t="inlineStr">
         <is>
           <t>予備1個購入→搭載（R12降ろす）</t>
         </is>
       </c>
+      <c r="R11" s="12" t="n"/>
       <c r="S11" s="12" t="n"/>
       <c r="T11" s="12" t="n"/>
     </row>
@@ -2213,19 +2227,19 @@
         <v>12</v>
       </c>
       <c r="O12" s="36" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="P12" s="36" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="Q12" s="36" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="R12" s="36" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="S12" s="36" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="T12" s="12" t="n"/>
     </row>
@@ -2255,13 +2269,13 @@
         <v>3</v>
       </c>
       <c r="I13" s="38" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="J13" s="38" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="K13" s="38" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="L13" s="38" t="n">
         <v>9</v>
@@ -2279,13 +2293,13 @@
         <v>12</v>
       </c>
       <c r="Q13" s="38" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="R13" s="38" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="S13" s="38" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="T13" s="12" t="n"/>
     </row>
@@ -2332,17 +2346,17 @@
       <c r="N14" s="40" t="n">
         <v>0</v>
       </c>
-      <c r="O14" s="41" t="n">
+      <c r="O14" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="P14" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q14" s="41" t="n">
         <v>1</v>
       </c>
-      <c r="P14" s="40" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q14" s="40" t="n">
-        <v>0</v>
-      </c>
-      <c r="R14" s="41" t="n">
-        <v>1</v>
+      <c r="R14" s="40" t="n">
+        <v>0</v>
       </c>
       <c r="S14" s="40" t="n">
         <v>0</v>
@@ -2380,7 +2394,7 @@
       </c>
       <c r="I15" s="12" t="n"/>
       <c r="J15" s="12" t="n"/>
-      <c r="K15" s="32" t="inlineStr">
+      <c r="K15" s="33" t="inlineStr">
         <is>
           <t>予備1個購入→搭載（R3降ろす）</t>
         </is>
@@ -2388,27 +2402,27 @@
       <c r="L15" s="31" t="inlineStr">
         <is>
           <t>機器更新（車両更新・電池2個付属）
-新品1個を救2へ／旧本体R11を救4へ</t>
+新品1個を救2へ／旧本体R11を救1へ</t>
         </is>
       </c>
       <c r="M15" s="12" t="n"/>
-      <c r="N15" s="33" t="inlineStr">
-        <is>
-          <t>救4更新の新品1個を受領（R8降ろす）</t>
-        </is>
-      </c>
-      <c r="O15" s="12" t="n"/>
+      <c r="N15" s="12" t="n"/>
+      <c r="O15" s="33" t="inlineStr">
+        <is>
+          <t>予備1個購入→搭載（R8降ろす）</t>
+        </is>
+      </c>
       <c r="P15" s="43" t="inlineStr">
         <is>
           <t>保守点検（新品1個）→救1へ</t>
         </is>
       </c>
-      <c r="Q15" s="32" t="inlineStr">
+      <c r="Q15" s="12" t="n"/>
+      <c r="R15" s="33" t="inlineStr">
         <is>
           <t>予備1個購入→搭載（R12降ろす）</t>
         </is>
       </c>
-      <c r="R15" s="12" t="n"/>
       <c r="S15" s="12" t="n"/>
       <c r="T15" s="12" t="n"/>
     </row>
@@ -2453,22 +2467,22 @@
         <v>12</v>
       </c>
       <c r="N16" s="36" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="O16" s="36" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="P16" s="36" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="Q16" s="36" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="R16" s="36" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="S16" s="36" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="T16" s="12" t="n"/>
     </row>
@@ -2513,7 +2527,7 @@
         <v>8</v>
       </c>
       <c r="N17" s="38" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="O17" s="38" t="n">
         <v>12</v>
@@ -2522,13 +2536,13 @@
         <v>12</v>
       </c>
       <c r="Q17" s="38" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="R17" s="38" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="S17" s="38" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="T17" s="12" t="n"/>
     </row>
@@ -2575,17 +2589,17 @@
       <c r="N18" s="40" t="n">
         <v>0</v>
       </c>
-      <c r="O18" s="40" t="n">
-        <v>0</v>
+      <c r="O18" s="41" t="n">
+        <v>1</v>
       </c>
       <c r="P18" s="40" t="n">
         <v>0</v>
       </c>
-      <c r="Q18" s="41" t="n">
+      <c r="Q18" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="R18" s="41" t="n">
         <v>1</v>
-      </c>
-      <c r="R18" s="40" t="n">
-        <v>0</v>
       </c>
       <c r="S18" s="40" t="n">
         <v>0</v>
@@ -2619,32 +2633,45 @@
           <t>保守点検（新品1個）</t>
         </is>
       </c>
-      <c r="G19" s="10" t="n"/>
+      <c r="G19" s="32" t="inlineStr">
+        <is>
+          <t>本体を救1へ載せ替え
+以降R8まで積載なし</t>
+        </is>
+      </c>
       <c r="H19" s="10" t="n"/>
-      <c r="I19" s="33" t="inlineStr">
-        <is>
-          <t>救2の新品1個とR6を交換</t>
-        </is>
-      </c>
-      <c r="J19" s="12" t="n"/>
+      <c r="I19" s="31" t="inlineStr">
+        <is>
+          <t>旧救2本体を受領（電池R3・R7付き）</t>
+        </is>
+      </c>
+      <c r="J19" s="33" t="inlineStr">
+        <is>
+          <t>予備1個購入→搭載（R3降ろす）</t>
+        </is>
+      </c>
       <c r="K19" s="12" t="n"/>
-      <c r="L19" s="33" t="inlineStr">
-        <is>
-          <t>旧救3本体のR11を受領（R3降ろす）</t>
-        </is>
-      </c>
-      <c r="M19" s="12" t="n"/>
+      <c r="L19" s="12" t="n"/>
+      <c r="M19" s="32" t="inlineStr">
+        <is>
+          <t>救2保守点検の新品を搭載（R7降ろす）</t>
+        </is>
+      </c>
       <c r="N19" s="31" t="inlineStr">
         <is>
           <t>機器更新（車両更新・電池2個付属）
-新品1個を救3へ／旧本体R11を継続搭載</t>
-        </is>
-      </c>
-      <c r="O19" s="12" t="n"/>
+旧本体R13を救1へ</t>
+        </is>
+      </c>
+      <c r="O19" s="32" t="inlineStr">
+        <is>
+          <t>新品予備1個を救2へ／救2のR9を受領</t>
+        </is>
+      </c>
       <c r="P19" s="12" t="n"/>
       <c r="Q19" s="43" t="inlineStr">
         <is>
-          <t>保守点検（新品1個）</t>
+          <t>保守点検（新品1個）（R9降ろす）</t>
         </is>
       </c>
       <c r="R19" s="12" t="n"/>
@@ -2670,26 +2697,22 @@
       <c r="F20" s="35" t="n">
         <v>6</v>
       </c>
-      <c r="G20" s="35" t="n">
-        <v>6</v>
-      </c>
-      <c r="H20" s="35" t="n">
-        <v>6</v>
-      </c>
+      <c r="G20" s="35" t="n"/>
+      <c r="H20" s="35" t="n"/>
       <c r="I20" s="36" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="J20" s="36" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="K20" s="36" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="L20" s="36" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="M20" s="36" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="N20" s="36" t="n">
         <v>14</v>
@@ -2730,35 +2753,31 @@
       <c r="F21" s="37" t="n">
         <v>3</v>
       </c>
-      <c r="G21" s="37" t="n">
-        <v>3</v>
-      </c>
-      <c r="H21" s="37" t="n">
-        <v>3</v>
-      </c>
+      <c r="G21" s="37" t="n"/>
+      <c r="H21" s="37" t="n"/>
       <c r="I21" s="38" t="n">
         <v>3</v>
       </c>
       <c r="J21" s="38" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="K21" s="38" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="L21" s="38" t="n">
+        <v>7</v>
+      </c>
+      <c r="M21" s="38" t="n">
+        <v>10</v>
+      </c>
+      <c r="N21" s="38" t="n">
+        <v>14</v>
+      </c>
+      <c r="O21" s="38" t="n">
         <v>9</v>
       </c>
-      <c r="M21" s="38" t="n">
+      <c r="P21" s="38" t="n">
         <v>9</v>
-      </c>
-      <c r="N21" s="38" t="n">
-        <v>11</v>
-      </c>
-      <c r="O21" s="38" t="n">
-        <v>11</v>
-      </c>
-      <c r="P21" s="38" t="n">
-        <v>11</v>
       </c>
       <c r="Q21" s="38" t="n">
         <v>14</v>
@@ -2799,8 +2818,8 @@
       <c r="I22" s="40" t="n">
         <v>0</v>
       </c>
-      <c r="J22" s="40" t="n">
-        <v>0</v>
+      <c r="J22" s="41" t="n">
+        <v>1</v>
       </c>
       <c r="K22" s="40" t="n">
         <v>0</v>
@@ -3206,7 +3225,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>元資料「保守点検及び本体、バッテリ更新計画（2026.5修正）」の機器更新・保守点検スケジュールはそのまま、R9以降の予備バッテリ購入数のみ精査したもの。</t>
+          <t>元資料「保守点検及び本体、バッテリ更新計画（2026.5修正）」をベースに、①R7の救急犬山1の車両更新（ルーカスは購入せず救急犬山4の本体を載せ替え）、②救急犬山2の旧本体の載せ替え先は救急犬山4、の2点を反映し、R9以降の予備バッテリ購入数を精査したもの。機器更新・保守点検の年度は元資料から変更していない。</t>
         </is>
       </c>
     </row>
@@ -3404,32 +3423,37 @@
       <c r="D7" s="10" t="n"/>
       <c r="E7" s="10" t="n"/>
       <c r="F7" s="10" t="n"/>
-      <c r="G7" s="10" t="n"/>
+      <c r="G7" s="31" t="inlineStr">
+        <is>
+          <t>車両更新（ルーカス購入なし）
+救4の本体を載せ替え（電池R3・R6も）</t>
+        </is>
+      </c>
       <c r="H7" s="10" t="n"/>
-      <c r="I7" s="31" t="inlineStr">
-        <is>
-          <t>旧救2本体を引継（電池R7・R3も引継）</t>
-        </is>
-      </c>
-      <c r="J7" s="12" t="n"/>
-      <c r="K7" s="32" t="inlineStr">
-        <is>
-          <t>予備1個購入→搭載（R3降ろす）</t>
-        </is>
-      </c>
-      <c r="L7" s="12" t="n"/>
+      <c r="I7" s="12" t="n"/>
+      <c r="J7" s="32" t="inlineStr">
+        <is>
+          <t>救2の新品1個を受領（R3降ろす）</t>
+        </is>
+      </c>
+      <c r="K7" s="12" t="n"/>
+      <c r="L7" s="32" t="inlineStr">
+        <is>
+          <t>救3更新の新品1個を受領（R6降ろす）</t>
+        </is>
+      </c>
       <c r="M7" s="12" t="n"/>
-      <c r="N7" s="33" t="inlineStr">
-        <is>
-          <t>救4更新の新品1個を受領（R7降ろす）</t>
+      <c r="N7" s="32" t="inlineStr">
+        <is>
+          <t>救4更新の新品1個を受領（R9降ろす）</t>
         </is>
       </c>
       <c r="O7" s="12" t="n"/>
       <c r="P7" s="12" t="n"/>
       <c r="Q7" s="12" t="n"/>
-      <c r="R7" s="32" t="inlineStr">
-        <is>
-          <t>予備1個購入→搭載（R11降ろす）</t>
+      <c r="R7" s="33" t="inlineStr">
+        <is>
+          <t>予備1個購入→搭載（R12降ろす）</t>
         </is>
       </c>
       <c r="S7" s="12" t="n"/>
@@ -3446,22 +3470,26 @@
       <c r="D8" s="35" t="n"/>
       <c r="E8" s="35" t="n"/>
       <c r="F8" s="35" t="n"/>
-      <c r="G8" s="35" t="n"/>
-      <c r="H8" s="35" t="n"/>
+      <c r="G8" s="35" t="n">
+        <v>6</v>
+      </c>
+      <c r="H8" s="35" t="n">
+        <v>6</v>
+      </c>
       <c r="I8" s="36" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="J8" s="36" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="K8" s="36" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="L8" s="36" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="M8" s="36" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="N8" s="36" t="n">
         <v>14</v>
@@ -3494,34 +3522,38 @@
       <c r="D9" s="37" t="n"/>
       <c r="E9" s="37" t="n"/>
       <c r="F9" s="37" t="n"/>
-      <c r="G9" s="37" t="n"/>
-      <c r="H9" s="37" t="n"/>
+      <c r="G9" s="37" t="n">
+        <v>3</v>
+      </c>
+      <c r="H9" s="37" t="n">
+        <v>3</v>
+      </c>
       <c r="I9" s="38" t="n">
         <v>3</v>
       </c>
       <c r="J9" s="38" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="K9" s="38" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="L9" s="38" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="M9" s="38" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="N9" s="38" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="O9" s="38" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="P9" s="38" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="Q9" s="38" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="R9" s="38" t="n">
         <v>14</v>
@@ -3562,8 +3594,8 @@
       <c r="J10" s="40" t="n">
         <v>0</v>
       </c>
-      <c r="K10" s="41" t="n">
-        <v>1</v>
+      <c r="K10" s="40" t="n">
+        <v>0</v>
       </c>
       <c r="L10" s="40" t="n">
         <v>0</v>
@@ -3622,25 +3654,26 @@
       <c r="H11" s="10" t="n"/>
       <c r="I11" s="31" t="inlineStr">
         <is>
-          <t>機器更新（車両更新・電池2個付属）</t>
-        </is>
-      </c>
-      <c r="J11" s="33" t="inlineStr">
-        <is>
-          <t>新品1個を救4のR6と交換</t>
+          <t>機器更新（車両更新・電池2個付属）
+旧本体を救4へ</t>
+        </is>
+      </c>
+      <c r="J11" s="32" t="inlineStr">
+        <is>
+          <t>新品1個を救1のR3と交換</t>
         </is>
       </c>
       <c r="K11" s="12" t="n"/>
       <c r="L11" s="12" t="n"/>
       <c r="M11" s="43" t="inlineStr">
         <is>
-          <t>保守点検（新品1個）（R6降ろす）</t>
+          <t>保守点検（新品1個）（R3降ろす）</t>
         </is>
       </c>
       <c r="N11" s="12" t="n"/>
       <c r="O11" s="12" t="n"/>
       <c r="P11" s="12" t="n"/>
-      <c r="Q11" s="33" t="inlineStr">
+      <c r="Q11" s="32" t="inlineStr">
         <is>
           <t>救4保守点検の新品を搭載（R9降ろす）</t>
         </is>
@@ -3738,13 +3771,13 @@
         <v>9</v>
       </c>
       <c r="J13" s="38" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="K13" s="38" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="L13" s="38" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="M13" s="38" t="n">
         <v>9</v>
@@ -3864,19 +3897,15 @@
       <c r="L15" s="31" t="inlineStr">
         <is>
           <t>機器更新（車両更新・電池2個付属）
-旧本体R8を救4へ</t>
-        </is>
-      </c>
-      <c r="M15" s="33" t="inlineStr">
-        <is>
-          <t>新品R12と救4のR9を交換</t>
-        </is>
-      </c>
+新品1個を救1へ／旧本体R8を継続搭載</t>
+        </is>
+      </c>
+      <c r="M15" s="12" t="n"/>
       <c r="N15" s="12" t="n"/>
       <c r="O15" s="12" t="n"/>
       <c r="P15" s="43" t="inlineStr">
         <is>
-          <t>保守点検（新品1個）（R9降ろす）</t>
+          <t>保守点検（新品1個）（R8降ろす）</t>
         </is>
       </c>
       <c r="Q15" s="12" t="n"/>
@@ -3979,16 +4008,16 @@
         <v>3</v>
       </c>
       <c r="L17" s="38" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="M17" s="38" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="N17" s="38" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="O17" s="38" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="P17" s="38" t="n">
         <v>12</v>
@@ -4091,29 +4120,30 @@
           <t>保守点検（新品1個）</t>
         </is>
       </c>
-      <c r="G19" s="10" t="n"/>
+      <c r="G19" s="32" t="inlineStr">
+        <is>
+          <t>本体を救1へ載せ替え
+以降R8まで積載なし</t>
+        </is>
+      </c>
       <c r="H19" s="10" t="n"/>
-      <c r="I19" s="12" t="n"/>
-      <c r="J19" s="33" t="inlineStr">
-        <is>
-          <t>救2の新品1個とR6を交換</t>
-        </is>
-      </c>
-      <c r="K19" s="12" t="n"/>
-      <c r="L19" s="33" t="inlineStr">
-        <is>
-          <t>旧救3本体のR8を受領（R3降ろす）</t>
-        </is>
-      </c>
-      <c r="M19" s="33" t="inlineStr">
-        <is>
-          <t>救3のR12とR9を交換</t>
-        </is>
-      </c>
+      <c r="I19" s="31" t="inlineStr">
+        <is>
+          <t>旧救2本体を受領（電池R3・R7付き）</t>
+        </is>
+      </c>
+      <c r="J19" s="12" t="n"/>
+      <c r="K19" s="33" t="inlineStr">
+        <is>
+          <t>予備1個購入→搭載（R3降ろす）</t>
+        </is>
+      </c>
+      <c r="L19" s="12" t="n"/>
+      <c r="M19" s="12" t="n"/>
       <c r="N19" s="31" t="inlineStr">
         <is>
           <t>機器更新（車両更新・電池2個付属）
-新品1個を救1へ／旧本体R12を継続搭載</t>
+新品1個を救1へ／旧本体R11を継続搭載</t>
         </is>
       </c>
       <c r="O19" s="12" t="n"/>
@@ -4123,9 +4153,9 @@
           <t>保守点検（新品1個）→救2へ</t>
         </is>
       </c>
-      <c r="R19" s="32" t="inlineStr">
-        <is>
-          <t>予備1個購入→搭載（R12降ろす）</t>
+      <c r="R19" s="33" t="inlineStr">
+        <is>
+          <t>予備1個購入→搭載（R11降ろす）</t>
         </is>
       </c>
       <c r="S19" s="12" t="n"/>
@@ -4150,26 +4180,22 @@
       <c r="F20" s="35" t="n">
         <v>6</v>
       </c>
-      <c r="G20" s="35" t="n">
-        <v>6</v>
-      </c>
-      <c r="H20" s="35" t="n">
-        <v>6</v>
-      </c>
+      <c r="G20" s="35" t="n"/>
+      <c r="H20" s="35" t="n"/>
       <c r="I20" s="36" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="J20" s="36" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="K20" s="36" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="L20" s="36" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="M20" s="36" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="N20" s="36" t="n">
         <v>14</v>
@@ -4210,12 +4236,8 @@
       <c r="F21" s="37" t="n">
         <v>3</v>
       </c>
-      <c r="G21" s="37" t="n">
-        <v>3</v>
-      </c>
-      <c r="H21" s="37" t="n">
-        <v>3</v>
-      </c>
+      <c r="G21" s="37" t="n"/>
+      <c r="H21" s="37" t="n"/>
       <c r="I21" s="38" t="n">
         <v>3</v>
       </c>
@@ -4223,25 +4245,25 @@
         <v>3</v>
       </c>
       <c r="K21" s="38" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="L21" s="38" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="M21" s="38" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="N21" s="38" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="O21" s="38" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="P21" s="38" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="Q21" s="38" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="R21" s="38" t="n">
         <v>14</v>
@@ -4282,8 +4304,8 @@
       <c r="J22" s="40" t="n">
         <v>0</v>
       </c>
-      <c r="K22" s="40" t="n">
-        <v>0</v>
+      <c r="K22" s="41" t="n">
+        <v>1</v>
       </c>
       <c r="L22" s="40" t="n">
         <v>0</v>
@@ -4651,7 +4673,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D35"/>
+  <dimension ref="A1:D37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -4712,7 +4734,7 @@
       </c>
       <c r="B6" s="59" t="inlineStr">
         <is>
-          <t>救2の新品1個と救4のR6を交換</t>
+          <t>救2機器更新。旧救2本体（電池R3・R7）を救4へ載せ替え／救2の新品1個と救1のR3を交換</t>
         </is>
       </c>
       <c r="C6" s="12" t="n">
@@ -4730,7 +4752,7 @@
       </c>
       <c r="B7" s="59" t="inlineStr">
         <is>
-          <t>1個購入 → 救1に搭載</t>
+          <t>1個購入 → 救4に搭載（R3を降ろす）</t>
         </is>
       </c>
       <c r="C7" s="11" t="n">
@@ -4748,7 +4770,7 @@
       </c>
       <c r="B8" s="59" t="inlineStr">
         <is>
-          <t>1個購入 → 救3に搭載</t>
+          <t>1個購入 → 救3に搭載（R3を降ろす）</t>
         </is>
       </c>
       <c r="C8" s="11" t="n">
@@ -4766,7 +4788,7 @@
       </c>
       <c r="B9" s="59" t="inlineStr">
         <is>
-          <t>救3更新の新品1個 → 救2へ／旧救3本体のR11 → 救4へ</t>
+          <t>救3機器更新。新品1個 → 救2へ／旧救3本体のR11 → 救1へ</t>
         </is>
       </c>
       <c r="C9" s="12" t="n">
@@ -4784,7 +4806,7 @@
       </c>
       <c r="B10" s="59" t="inlineStr">
         <is>
-          <t>救2保守点検の新品 → 救1へ</t>
+          <t>救2保守点検の新品 → 救4へ</t>
         </is>
       </c>
       <c r="C10" s="12" t="n">
@@ -4802,7 +4824,7 @@
       </c>
       <c r="B11" s="59" t="inlineStr">
         <is>
-          <t>救4更新の新品1個 → 救3へ</t>
+          <t>救4機器更新。旧救4本体のR13 → 救1へ</t>
         </is>
       </c>
       <c r="C11" s="12" t="n">
@@ -4820,7 +4842,7 @@
       </c>
       <c r="B12" s="59" t="inlineStr">
         <is>
-          <t>1個購入 → 救2に搭載</t>
+          <t>救4の新品予備1個 → 救2へ（救2のR9を救4へ）／1個購入 → 救3に搭載</t>
         </is>
       </c>
       <c r="C12" s="11" t="n">
@@ -4856,7 +4878,7 @@
       </c>
       <c r="B14" s="59" t="inlineStr">
         <is>
-          <t>1個購入 → 救3に搭載</t>
+          <t>救4保守点検（新品1個）／1個購入 → 救2に搭載</t>
         </is>
       </c>
       <c r="C14" s="11" t="n">
@@ -4874,7 +4896,7 @@
       </c>
       <c r="B15" s="59" t="inlineStr">
         <is>
-          <t>1個購入 → 救2に搭載</t>
+          <t>1個購入 → 救3に搭載</t>
         </is>
       </c>
       <c r="C15" s="11" t="n">
@@ -4955,7 +4977,7 @@
       </c>
       <c r="B22" s="59" t="inlineStr">
         <is>
-          <t>作業なし（救2の機器更新で新品2個が入るため）</t>
+          <t>救2機器更新。旧救2本体（電池R3・R7）を救4へ載せ替え（購入なし）</t>
         </is>
       </c>
       <c r="C22" s="12" t="n">
@@ -4963,7 +4985,7 @@
       </c>
       <c r="D22" s="40" t="inlineStr">
         <is>
-          <t>購入なし</t>
+          <t>入替のみ（購入なし）</t>
         </is>
       </c>
     </row>
@@ -4973,7 +4995,7 @@
       </c>
       <c r="B23" s="59" t="inlineStr">
         <is>
-          <t>救2の新品1個と救4のR6を交換</t>
+          <t>救2の新品1個と救1のR3を交換</t>
         </is>
       </c>
       <c r="C23" s="12" t="n">
@@ -4991,7 +5013,7 @@
       </c>
       <c r="B24" s="59" t="inlineStr">
         <is>
-          <t>1個購入 → 救1に搭載</t>
+          <t>1個購入 → 救4に搭載（R3を降ろす）</t>
         </is>
       </c>
       <c r="C24" s="11" t="n">
@@ -5009,7 +5031,7 @@
       </c>
       <c r="B25" s="59" t="inlineStr">
         <is>
-          <t>旧救3本体のR8 → 救4へ</t>
+          <t>救3機器更新。新品1個 → 救1へ（救1のR6を降ろす）</t>
         </is>
       </c>
       <c r="C25" s="12" t="n">
@@ -5027,7 +5049,7 @@
       </c>
       <c r="B26" s="59" t="inlineStr">
         <is>
-          <t>救3のR12と救4のR9を交換</t>
+          <t>救2保守点検（新品1個）</t>
         </is>
       </c>
       <c r="C26" s="12" t="n">
@@ -5045,7 +5067,7 @@
       </c>
       <c r="B27" s="59" t="inlineStr">
         <is>
-          <t>救4更新の新品1個 → 救1へ</t>
+          <t>救4機器更新。新品1個 → 救1へ（救1のR9を降ろす）</t>
         </is>
       </c>
       <c r="C27" s="12" t="n">
@@ -5059,69 +5081,94 @@
     </row>
     <row r="28">
       <c r="A28" s="58" t="n">
+        <v>16</v>
+      </c>
+      <c r="B28" s="59" t="inlineStr">
+        <is>
+          <t>救3保守点検（新品1個）</t>
+        </is>
+      </c>
+      <c r="C28" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="D28" s="40" t="inlineStr">
+        <is>
+          <t>入替のみ（購入なし）</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="58" t="n">
         <v>17</v>
       </c>
-      <c r="B28" s="59" t="inlineStr">
+      <c r="B29" s="59" t="inlineStr">
         <is>
           <t>救4保守点検の新品 → 救2へ</t>
         </is>
       </c>
-      <c r="C28" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="D28" s="40" t="inlineStr">
+      <c r="C29" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="D29" s="40" t="inlineStr">
         <is>
           <t>入替のみ（購入なし）</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="60" t="n">
+    <row r="30">
+      <c r="A30" s="60" t="n">
         <v>18</v>
       </c>
-      <c r="B29" s="59" t="inlineStr">
+      <c r="B30" s="59" t="inlineStr">
         <is>
           <t>2個購入 → 救1・救4に搭載</t>
         </is>
       </c>
-      <c r="C29" s="11" t="n">
+      <c r="C30" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="D29" s="40" t="inlineStr">
+      <c r="D30" s="40" t="inlineStr">
         <is>
           <t>購入あり</t>
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="42" t="inlineStr">
+    <row r="31">
+      <c r="A31" s="42" t="inlineStr">
         <is>
           <t>合計</t>
         </is>
       </c>
-      <c r="B30" s="45" t="inlineStr"/>
-      <c r="C30" s="13">
-        <f>SUM(C22:C29)</f>
-        <v/>
-      </c>
-      <c r="D30" s="45" t="inlineStr"/>
-    </row>
-    <row r="33">
-      <c r="A33" s="2" t="inlineStr">
-        <is>
-          <t>※ R9は両案とも購入0個。救急犬山2の機器更新で新品バッテリ2個が入るため。</t>
-        </is>
-      </c>
+      <c r="B31" s="45" t="inlineStr"/>
+      <c r="C31" s="13">
+        <f>SUM(C22:C30)</f>
+        <v/>
+      </c>
+      <c r="D31" s="45" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>※ 「交換」は2台の車の間で電池を入れ替えること。「→○○へ」は付属してきた新品を別の車に回すこと。</t>
+          <t>※ R9は両案とも購入0個。救急犬山2の機器更新で新品バッテリ2個が入るため。</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>※ R7（実績）に救急犬山1の車両更新があり、ルーカスは購入せず救急犬山4の本体を載せ替えている。救急犬山4はR9に旧救急犬山2本体を受領するまで積載なし。</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>※ 「交換」は2台の車の間で電池を入れ替えること。「→○○へ」は付属してきた新品を別の車に回すこと。</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
         <is>
           <t>※ 機器更新で外した旧本体に付いていた電池は、新本体で使用できるか事前にメーカーへ要確認。</t>
         </is>
@@ -5142,7 +5189,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D44"/>
+  <dimension ref="A1:D47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -5358,7 +5405,7 @@
     <row r="21">
       <c r="A21" s="55" t="inlineStr">
         <is>
-          <t>4．元資料（2026.5修正）の機器スケジュール　※本計画では変更していない</t>
+          <t>4．機器スケジュール　※年度は元資料（2026.5修正）のまま。載せ替え先のみ修正</t>
         </is>
       </c>
       <c r="B21" s="56" t="n"/>
@@ -5394,17 +5441,17 @@
       </c>
       <c r="B23" s="12" t="inlineStr">
         <is>
-          <t>―（R9に旧救2本体を引継）</t>
+          <t>―</t>
         </is>
       </c>
       <c r="C23" s="12" t="inlineStr">
         <is>
-          <t>―</t>
+          <t>―（元資料に記載なし）</t>
         </is>
       </c>
       <c r="D23" s="12" t="inlineStr">
         <is>
-          <t>―（元資料に記載なし）</t>
+          <t>R7　車両更新。ルーカスは購入せず救4の本体を載せ替え</t>
         </is>
       </c>
     </row>
@@ -5426,7 +5473,7 @@
       </c>
       <c r="D24" s="12" t="inlineStr">
         <is>
-          <t>R9</t>
+          <t>R9　旧本体は救4へ載せ替え</t>
         </is>
       </c>
     </row>
@@ -5470,7 +5517,7 @@
       </c>
       <c r="D26" s="12" t="inlineStr">
         <is>
-          <t>R14</t>
+          <t>R14　※R7〜R8は積載なし、R9に旧救2本体を受領</t>
         </is>
       </c>
     </row>
@@ -5535,7 +5582,7 @@
     <row r="35">
       <c r="A35" s="59" t="inlineStr">
         <is>
-          <t>・R9に、旧救急犬山2本体（R7とR3のバッテリ付き）を救急犬山1へ積載する。</t>
+          <t>・R7に救急犬山1の車両更新。ルーカス本体は購入せず、救急犬山4の本体（バッテリR3・R6付き）を救急犬山1へ載せ替える。</t>
         </is>
       </c>
       <c r="B35" s="56" t="n"/>
@@ -5545,7 +5592,7 @@
     <row r="36">
       <c r="A36" s="59" t="inlineStr">
         <is>
-          <t>・機器更新で外した旧本体のバッテリは、他の車で再利用する。</t>
+          <t>・R7〜R8の間、救急犬山4は積載なし（この期間はバッテリ計画の対象外）。</t>
         </is>
       </c>
       <c r="B36" s="56" t="n"/>
@@ -5555,7 +5602,7 @@
     <row r="37">
       <c r="A37" s="59" t="inlineStr">
         <is>
-          <t>・救急犬山1の本体更新は元資料に記載がないため、本計画には含めていない。</t>
+          <t>・R9に、旧救急犬山2本体（バッテリR3・R7付き）を救急犬山4へ載せ替える。</t>
         </is>
       </c>
       <c r="B37" s="56" t="n"/>
@@ -5565,46 +5612,46 @@
     <row r="38">
       <c r="A38" s="59" t="inlineStr">
         <is>
-          <t>・R3〜R8は実績として扱い、購入計画はR9（令和9年度）以降を対象とする。</t>
+          <t>・機器更新で外した旧本体のバッテリは、他の車で再利用する。</t>
         </is>
       </c>
       <c r="B38" s="56" t="n"/>
       <c r="C38" s="56" t="n"/>
       <c r="D38" s="57" t="n"/>
     </row>
+    <row r="39">
+      <c r="A39" s="59" t="inlineStr">
+        <is>
+          <t>・救急犬山1の本体更新は元資料に記載がないため、本計画には含めていない。</t>
+        </is>
+      </c>
+      <c r="B39" s="56" t="n"/>
+      <c r="C39" s="56" t="n"/>
+      <c r="D39" s="57" t="n"/>
+    </row>
     <row r="40">
-      <c r="A40" s="55" t="inlineStr">
+      <c r="A40" s="59" t="inlineStr">
+        <is>
+          <t>・R3〜R8は実績として扱い、購入計画はR9（令和9年度）以降を対象とする。</t>
+        </is>
+      </c>
+      <c r="B40" s="56" t="n"/>
+      <c r="C40" s="56" t="n"/>
+      <c r="D40" s="57" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="55" t="inlineStr">
         <is>
           <t>7．要確認事項</t>
         </is>
       </c>
-      <c r="B40" s="56" t="n"/>
-      <c r="C40" s="57" t="n"/>
-    </row>
-    <row r="41" ht="28" customHeight="1">
-      <c r="A41" s="62" t="inlineStr">
-        <is>
-          <t>・旧本体から外したバッテリが新本体でそのまま使用できるか（メーカー確認）。</t>
-        </is>
-      </c>
-      <c r="B41" s="56" t="n"/>
-      <c r="C41" s="56" t="n"/>
-      <c r="D41" s="57" t="n"/>
-    </row>
-    <row r="42" ht="28" customHeight="1">
-      <c r="A42" s="62" t="inlineStr">
-        <is>
-          <t>・救急犬山1の本体は R3配備（旧救2）のため、耐用期間8年は R11 に到達する。R11以降の本体の取扱い（救3・救4の旧本体を回すか等）は元資料に記載がなく、別途検討が必要。</t>
-        </is>
-      </c>
       <c r="B42" s="56" t="n"/>
-      <c r="C42" s="56" t="n"/>
-      <c r="D42" s="57" t="n"/>
+      <c r="C42" s="57" t="n"/>
     </row>
     <row r="43" ht="28" customHeight="1">
       <c r="A43" s="62" t="inlineStr">
         <is>
-          <t>・車両間でバッテリを入れ替える運用が可能か（管理簿・資器材管理上の取扱い）。</t>
+          <t>・旧本体から外したバッテリが新本体でそのまま使用できるか（メーカー確認）。</t>
         </is>
       </c>
       <c r="B43" s="56" t="n"/>
@@ -5614,33 +5661,66 @@
     <row r="44" ht="28" customHeight="1">
       <c r="A44" s="62" t="inlineStr">
         <is>
-          <t>・入替を行わない場合は、比較まとめシートの「参考」行（3年版12個／4年版5個）となる。</t>
+          <t>・救急犬山1の本体は R3配備（旧救4）のため、耐用期間8年は R11 に到達する。R11以降の本体の取扱い（救3・救4の旧本体を回すか等）は元資料に記載がなく、別途検討が必要。</t>
         </is>
       </c>
       <c r="B44" s="56" t="n"/>
       <c r="C44" s="56" t="n"/>
       <c r="D44" s="57" t="n"/>
     </row>
+    <row r="45" ht="28" customHeight="1">
+      <c r="A45" s="62" t="inlineStr">
+        <is>
+          <t>・救急犬山1には保守点検が組まれていない（元資料の表に記載がない）ため、本計画もそのまま組んでいる。点検を入れる場合は購入数が変わる。</t>
+        </is>
+      </c>
+      <c r="B45" s="56" t="n"/>
+      <c r="C45" s="56" t="n"/>
+      <c r="D45" s="57" t="n"/>
+    </row>
+    <row r="46" ht="28" customHeight="1">
+      <c r="A46" s="62" t="inlineStr">
+        <is>
+          <t>・車両間でバッテリを入れ替える運用が可能か（管理簿・資器材管理上の取扱い）。</t>
+        </is>
+      </c>
+      <c r="B46" s="56" t="n"/>
+      <c r="C46" s="56" t="n"/>
+      <c r="D46" s="57" t="n"/>
+    </row>
+    <row r="47" ht="28" customHeight="1">
+      <c r="A47" s="62" t="inlineStr">
+        <is>
+          <t>・入替を行わない場合は、比較まとめシートの「参考」行（3年版12個／4年版5個）となる。</t>
+        </is>
+      </c>
+      <c r="B47" s="56" t="n"/>
+      <c r="C47" s="56" t="n"/>
+      <c r="D47" s="57" t="n"/>
+    </row>
   </sheetData>
-  <mergeCells count="19">
+  <mergeCells count="22">
     <mergeCell ref="A35:D35"/>
     <mergeCell ref="A38:D38"/>
     <mergeCell ref="A29:D29"/>
     <mergeCell ref="A43:D43"/>
     <mergeCell ref="A21:C21"/>
     <mergeCell ref="A44:D44"/>
+    <mergeCell ref="A42:C42"/>
+    <mergeCell ref="A40:D40"/>
     <mergeCell ref="A31:D31"/>
     <mergeCell ref="A14:C14"/>
     <mergeCell ref="A8:C8"/>
     <mergeCell ref="A30:D30"/>
+    <mergeCell ref="A39:D39"/>
     <mergeCell ref="A4:C4"/>
     <mergeCell ref="A36:D36"/>
     <mergeCell ref="A28:C28"/>
-    <mergeCell ref="A40:C40"/>
-    <mergeCell ref="A41:D41"/>
+    <mergeCell ref="A45:D45"/>
     <mergeCell ref="A34:C34"/>
+    <mergeCell ref="A46:D46"/>
     <mergeCell ref="A37:D37"/>
-    <mergeCell ref="A42:D42"/>
+    <mergeCell ref="A47:D47"/>
     <mergeCell ref="A32:D32"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>